<commit_message>
Align verification template with order-level lookup columns
Treat order-line discounts as reference only. Fill activity amount when an order has activity redemption, coupon amount when it has a coupon, and leave gift quantity blank until configuration arrives.

Co-authored-by: peggyzhan1 <peggyzhan1@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/templates/活动费用核验报告模版.xlsx
+++ b/docs/templates/活动费用核验报告模版.xlsx
@@ -13,7 +13,7 @@
     <sheet name="字段说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'参与订单明细'!$A$2:$Y$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'参与订单明细'!$A$2:$AA$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'订单商品行（附录）'!$A$2:$J$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段说明'!$A$2:$F$2</definedName>
   </definedNames>
@@ -150,11 +150,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -915,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y5"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -936,19 +936,21 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>一行一张参与本活动的订单。活动优惠金额是计费列；橙色三列以后才填。</t>
+          <t>一行一张订单。订单优惠金额只备查；关联活动则填活动优惠金额，关联券则填券优惠，满赠则以后填满赠数量。</t>
         </is>
       </c>
     </row>
@@ -1045,35 +1047,45 @@
       </c>
       <c r="S2" s="9" t="inlineStr">
         <is>
+          <t>订单优惠金额（备查）</t>
+        </is>
+      </c>
+      <c r="T2" s="9" t="inlineStr">
+        <is>
           <t>活动优惠金额</t>
         </is>
       </c>
-      <c r="T2" s="9" t="inlineStr">
+      <c r="U2" s="9" t="inlineStr">
+        <is>
+          <t>优惠券优惠金额</t>
+        </is>
+      </c>
+      <c r="V2" s="10" t="inlineStr">
+        <is>
+          <t>满赠数量</t>
+        </is>
+      </c>
+      <c r="W2" s="9" t="inlineStr">
         <is>
           <t>是否可释放</t>
         </is>
       </c>
-      <c r="U2" s="9" t="inlineStr">
+      <c r="X2" s="9" t="inlineStr">
         <is>
           <t>释放结论</t>
         </is>
       </c>
-      <c r="V2" s="9" t="inlineStr">
-        <is>
-          <t>同单券优惠金额</t>
-        </is>
-      </c>
-      <c r="W2" s="10" t="inlineStr">
+      <c r="Y2" s="10" t="inlineStr">
         <is>
           <t>理论权益</t>
         </is>
       </c>
-      <c r="X2" s="10" t="inlineStr">
+      <c r="Z2" s="10" t="inlineStr">
         <is>
           <t>一致性</t>
         </is>
       </c>
-      <c r="Y2" s="10" t="inlineStr">
+      <c r="AA2" s="10" t="inlineStr">
         <is>
           <t>差异金额</t>
         </is>
@@ -1167,24 +1179,26 @@
         <v>1126.5</v>
       </c>
       <c r="S3" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="T3" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="T3" s="12" t="inlineStr">
+      <c r="U3" s="11" t="inlineStr"/>
+      <c r="V3" s="12" t="inlineStr"/>
+      <c r="W3" s="13" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="U3" s="11" t="inlineStr">
+      <c r="X3" s="11" t="inlineStr">
         <is>
           <t>已完成且达到T-2</t>
         </is>
       </c>
-      <c r="V3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="13" t="inlineStr"/>
-      <c r="X3" s="13" t="inlineStr"/>
-      <c r="Y3" s="13" t="inlineStr"/>
+      <c r="Y3" s="12" t="inlineStr"/>
+      <c r="Z3" s="12" t="inlineStr"/>
+      <c r="AA3" s="12" t="inlineStr"/>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="14" t="n">
@@ -1274,24 +1288,26 @@
         <v>331.82</v>
       </c>
       <c r="S4" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="T4" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="T4" s="12" t="inlineStr">
+      <c r="U4" s="14" t="inlineStr"/>
+      <c r="V4" s="12" t="inlineStr"/>
+      <c r="W4" s="13" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="U4" s="14" t="inlineStr">
+      <c r="X4" s="14" t="inlineStr">
         <is>
           <t>已完成且达到T-2</t>
         </is>
       </c>
-      <c r="V4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="13" t="inlineStr"/>
-      <c r="X4" s="13" t="inlineStr"/>
-      <c r="Y4" s="13" t="inlineStr"/>
+      <c r="Y4" s="12" t="inlineStr"/>
+      <c r="Z4" s="12" t="inlineStr"/>
+      <c r="AA4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="11" t="n">
@@ -1383,30 +1399,32 @@
       <c r="S5" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="T5" s="15" t="inlineStr">
+      <c r="T5" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="U5" s="11" t="inlineStr"/>
+      <c r="V5" s="12" t="inlineStr"/>
+      <c r="W5" s="15" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="U5" s="11" t="inlineStr">
+      <c r="X5" s="11" t="inlineStr">
         <is>
           <t>订单状态=部分发货</t>
         </is>
       </c>
-      <c r="V5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="13" t="inlineStr"/>
-      <c r="X5" s="13" t="inlineStr"/>
-      <c r="Y5" s="13" t="inlineStr"/>
+      <c r="Y5" s="12" t="inlineStr"/>
+      <c r="Z5" s="12" t="inlineStr"/>
+      <c r="AA5" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Y2"/>
+  <autoFilter ref="A2:AA2"/>
   <mergeCells count="1">
     <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="T3:T2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W3:W2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1719,7 +1737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2309,7 +2327,7 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>活动优惠金额</t>
+          <t>订单优惠金额（备查）</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -2319,12 +2337,12 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>activity_execution</t>
+          <t>order_line 合计</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>该单在本活动核销里的优惠，计费用这一列</t>
+          <t>订单明细优惠加总，只对照，不计本活动费用</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr"/>
@@ -2337,7 +2355,7 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>是否可释放</t>
+          <t>活动优惠金额</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -2347,12 +2365,12 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>release_candidate</t>
+          <t>activity_execution</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>是 / 否</t>
+          <t>关联了活动才有值；满减计费用这一列</t>
         </is>
       </c>
       <c r="F23" s="11" t="inlineStr"/>
@@ -2365,7 +2383,7 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>释放结论</t>
+          <t>优惠券优惠金额</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -2375,12 +2393,12 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>release_candidate</t>
+          <t>coupon_redemption</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>已完成且达到T-2，或不可释放原因</t>
+          <t>关联了券才有值，否则空</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr"/>
@@ -2393,22 +2411,22 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>同单券优惠金额</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>现在</t>
+          <t>满赠数量</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>以后</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>coupon_redemption</t>
+          <t>待核算引擎</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>该单若另有券核销，仅备查，不计入本活动费用</t>
+          <t>关联满赠才有值；现在空，配置进表后再填</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr"/>
@@ -2421,22 +2439,22 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>理论权益</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>以后</t>
+          <t>是否可释放</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>现在</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>待核算引擎</t>
+          <t>release_candidate</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>配置进标准表并改核算后填写，现在空</t>
+          <t>是 / 否</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr"/>
@@ -2449,22 +2467,22 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>一致性</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>以后</t>
+          <t>释放结论</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>现在</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>待核算引擎</t>
+          <t>release_candidate</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>理论与活动优惠比对，现在空</t>
+          <t>已完成且达到T-2，或不可释放原因</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr"/>
@@ -2477,10 +2495,10 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>差异金额</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
+          <t>理论权益</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>以后</t>
         </is>
@@ -2492,7 +2510,7 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>活动优惠 − 理论权益，现在空</t>
+          <t>配置进标准表并改核算后填写，现在空</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr"/>
@@ -2500,27 +2518,27 @@
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>订单商品行（附录）</t>
+          <t>参与订单明细</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>单据编号</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>现在</t>
+          <t>一致性</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>以后</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>order_header</t>
+          <t>待核算引擎</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>回指参与订单</t>
+          <t>理论与活动优惠比对，现在空</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr"/>
@@ -2528,27 +2546,27 @@
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>订单商品行（附录）</t>
+          <t>参与订单明细</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>商品编号</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>现在</t>
+          <t>差异金额</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>以后</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>order_line</t>
+          <t>待核算引擎</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>订单行</t>
+          <t>活动优惠 − 理论权益，现在空</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr"/>
@@ -2561,7 +2579,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>商品名称</t>
+          <t>单据编号</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -2571,12 +2589,12 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>order_line</t>
+          <t>order_header</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>订单行</t>
+          <t>回指参与订单</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr"/>
@@ -2589,7 +2607,7 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>规格</t>
+          <t>商品编号</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -2617,7 +2635,7 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>数量</t>
+          <t>商品名称</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
@@ -2645,7 +2663,7 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>单位</t>
+          <t>规格</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -2673,7 +2691,7 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>单价</t>
+          <t>数量</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
@@ -2701,7 +2719,7 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>折前金额</t>
+          <t>单位</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -2729,7 +2747,7 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>行优惠金额</t>
+          <t>单价</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
@@ -2744,7 +2762,7 @@
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>平台行分摊，只展示，不计入活动费用</t>
+          <t>订单行</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr"/>
@@ -2757,25 +2775,81 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
+          <t>折前金额</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>现在</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>order_line</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>订单行</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>订单商品行（附录）</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>行优惠金额</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>现在</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>order_line</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>平台行分摊，只展示，不计入活动费用</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>订单商品行（附录）</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
           <t>实付金额</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>现在</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>现在</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>order_line</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
+      <c r="E40" s="14" t="inlineStr">
         <is>
           <t>订单行</t>
         </is>
       </c>
-      <c r="F38" s="14" t="inlineStr"/>
+      <c r="F40" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:F2"/>

</xml_diff>